<commit_message>
finalized WBT TCs excel form
</commit_message>
<xml_diff>
--- a/docs/Lab03/Lab03_WBT_TCs_Form - AM03.xlsx
+++ b/docs/Lab03/Lab03_WBT_TCs_Form - AM03.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15AE3A50-9D07-4D74-844A-8F281F6F31F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAE1BCDF-C4F2-4371-AD41-CFD515BCAE9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="186">
   <si>
     <t>VVSS, Info Romana, 2025-2026</t>
   </si>
@@ -136,9 +136,6 @@
     <t>CC1 = No. of regions =</t>
   </si>
   <si>
-    <t>…</t>
-  </si>
-  <si>
     <t>Req02_L01</t>
   </si>
   <si>
@@ -157,9 +154,6 @@
     <t>Req02_L03</t>
   </si>
   <si>
-    <t>..</t>
-  </si>
-  <si>
     <t>F02. Individual Paths</t>
   </si>
   <si>
@@ -221,9 +215,6 @@
   </si>
   <si>
     <t>F02_TC01</t>
-  </si>
-  <si>
-    <t>F01_TC02</t>
   </si>
   <si>
     <t>WBT Implemented TCs</t>
@@ -830,18 +821,6 @@
     <t>1 - 2(F) - 4(T) - 5 - 6 - 7(F) - 4(F) - 12</t>
   </si>
   <si>
-    <t>F01_TC03</t>
-  </si>
-  <si>
-    <t>F01_TC04</t>
-  </si>
-  <si>
-    <t>F01_TC05</t>
-  </si>
-  <si>
-    <t>F01_TC06</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b/>
@@ -941,9 +920,6 @@
     <t>[sirop:20]</t>
   </si>
   <si>
-    <t>1;sirop devine 10 + 2;sirop neschimbat</t>
-  </si>
-  <si>
     <t>1, 2, 4, 5, 6, 7, 8, 9, 10, 11, 12</t>
   </si>
   <si>
@@ -962,9 +938,6 @@
     <t>sirop devine 20 + lapte devine 20</t>
   </si>
   <si>
-    <t>1;sirop;30;10, 2;sirop;50;10</t>
-  </si>
-  <si>
     <t>F02_TC03</t>
   </si>
   <si>
@@ -975,13 +948,91 @@
   </si>
   <si>
     <t>F02_TC06</t>
+  </si>
+  <si>
+    <t>Clasa de test</t>
+  </si>
+  <si>
+    <t>Metoda de test</t>
+  </si>
+  <si>
+    <t>StocServiceTest</t>
+  </si>
+  <si>
+    <t>consuma_douaIngrediente_consumaCorectPentruAmbele</t>
+  </si>
+  <si>
+    <t>execuție normală; espresso devine 20, lapte devine 20</t>
+  </si>
+  <si>
+    <t>PASS - espresso și lapte au devenit 20</t>
+  </si>
+  <si>
+    <t>PASS - primul stoc a devenit 30, al doilea a rămas 30</t>
+  </si>
+  <si>
+    <t>PASS - stocurile au devenit 0 și 10</t>
+  </si>
+  <si>
+    <t>PASS - espresso a devenit 50</t>
+  </si>
+  <si>
+    <t>PASS - stocul a rămas 50</t>
+  </si>
+  <si>
+    <t>PASS - IllegalStateException aruncată; stocul a rămas 50</t>
+  </si>
+  <si>
+    <t>IllegalStateException cu mesajul "Stoc insuficient pentru rețeta."</t>
+  </si>
+  <si>
+    <t>execuție normală; stoc neschimbat</t>
+  </si>
+  <si>
+    <t>execuție normală; espresso devine 50</t>
+  </si>
+  <si>
+    <t>execuție normală; primul lapte devine 0, al doilea devine 10</t>
+  </si>
+  <si>
+    <t>execuție normală; primul sirop devine 30, al doilea rămâne 30</t>
+  </si>
+  <si>
+    <t>consuma_ramasDevineZero_seExecutaBreak</t>
+  </si>
+  <si>
+    <t>consuma_unIngredient_douaPozitiiStoc_consumaDinAmbele</t>
+  </si>
+  <si>
+    <t>consuma_unIngredient_unSingurStoc_consumaCorect</t>
+  </si>
+  <si>
+    <t>consuma_retetaFaraIngrediente_nuModificaStocul</t>
+  </si>
+  <si>
+    <t>consuma_stocInsuficient_throwsException</t>
+  </si>
+  <si>
+    <t>1;lapte;30;10 | 2;lapte;50;10</t>
+  </si>
+  <si>
+    <t>1;sirop;50;10 | 2;sirop;30;10</t>
+  </si>
+  <si>
+    <t>1;sirop;50;10, 2;sirop;30;10</t>
+  </si>
+  <si>
+    <t>1;sirop devine 30 + 2;sirop neschimbat</t>
+  </si>
+  <si>
+    <t>1;sirop;50;10 | 2;lapte;60;10</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1226,7 +1277,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="63">
+  <borders count="64">
     <border>
       <left/>
       <right/>
@@ -2006,11 +2057,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="170">
+  <cellXfs count="172">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2082,264 +2144,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -2350,69 +2171,24 @@
     <xf numFmtId="0" fontId="14" fillId="5" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -2422,24 +2198,6 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2463,23 +2221,335 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="12" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2858,26 +2928,26 @@
     <tabColor theme="5" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="B1:P20"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="15" max="15" width="19.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:16">
       <c r="B1" s="11"/>
-      <c r="D1" s="35" t="s">
+      <c r="D1" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="37"/>
-    </row>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="67"/>
+    </row>
+    <row r="2" spans="2:16">
       <c r="B2" s="32" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:16">
       <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
@@ -2887,7 +2957,7 @@
       <c r="O4" s="5"/>
       <c r="P4" s="5"/>
     </row>
-    <row r="5" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:16">
       <c r="B5" s="1" t="s">
         <v>4</v>
       </c>
@@ -2897,7 +2967,7 @@
       <c r="O5" s="29"/>
       <c r="P5" s="29"/>
     </row>
-    <row r="6" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:16">
       <c r="B6" s="1" t="s">
         <v>6</v>
       </c>
@@ -2909,7 +2979,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:16">
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -2918,13 +2988,13 @@
         <v>9</v>
       </c>
       <c r="O7" s="23" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="P7" s="23">
         <v>235</v>
       </c>
     </row>
-    <row r="8" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:16">
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
@@ -2933,15 +3003,15 @@
         <v>10</v>
       </c>
       <c r="O8" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="P8" s="23">
         <v>235</v>
       </c>
     </row>
-    <row r="9" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:16">
       <c r="B9" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
@@ -2950,37 +3020,37 @@
         <v>11</v>
       </c>
       <c r="O9" s="23" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="P9" s="23">
         <v>235</v>
       </c>
     </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:16">
       <c r="B10" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
     </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:16">
       <c r="B11" s="30" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
     </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:16">
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:2">
       <c r="B19" s="1"/>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:2">
       <c r="B20" s="1"/>
     </row>
   </sheetData>
@@ -2998,7 +3068,7 @@
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="B1:W32"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="10" customWidth="1"/>
     <col min="5" max="5" width="8.88671875" customWidth="1"/>
@@ -3006,639 +3076,648 @@
     <col min="17" max="17" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:23" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:23">
       <c r="B1" s="11"/>
-      <c r="D1" s="35" t="s">
+      <c r="D1" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="37"/>
-    </row>
-    <row r="3" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B3" s="42" t="s">
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="67"/>
+    </row>
+    <row r="3" spans="2:23">
+      <c r="B3" s="83" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="43"/>
-      <c r="G3" s="43"/>
-      <c r="H3" s="43"/>
-      <c r="I3" s="43"/>
-      <c r="J3" s="43"/>
-      <c r="K3" s="44"/>
-    </row>
-    <row r="6" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B6" s="101" t="s">
+      <c r="C3" s="84"/>
+      <c r="D3" s="84"/>
+      <c r="E3" s="84"/>
+      <c r="F3" s="84"/>
+      <c r="G3" s="84"/>
+      <c r="H3" s="84"/>
+      <c r="I3" s="84"/>
+      <c r="J3" s="84"/>
+      <c r="K3" s="85"/>
+    </row>
+    <row r="6" spans="2:23">
+      <c r="B6" s="72" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="101"/>
-      <c r="D6" s="101"/>
-      <c r="E6" s="101"/>
-      <c r="F6" s="101"/>
-      <c r="G6" s="101"/>
-      <c r="H6" s="101"/>
-      <c r="I6" s="101"/>
-      <c r="K6" s="101" t="s">
+      <c r="C6" s="72"/>
+      <c r="D6" s="72"/>
+      <c r="E6" s="72"/>
+      <c r="F6" s="72"/>
+      <c r="G6" s="72"/>
+      <c r="H6" s="72"/>
+      <c r="I6" s="72"/>
+      <c r="K6" s="72" t="s">
         <v>14</v>
       </c>
-      <c r="L6" s="101"/>
-      <c r="M6" s="101"/>
-      <c r="N6" s="101"/>
-      <c r="O6" s="101"/>
-      <c r="P6" s="101"/>
-      <c r="Q6" s="101"/>
-      <c r="S6" s="101" t="s">
+      <c r="L6" s="72"/>
+      <c r="M6" s="72"/>
+      <c r="N6" s="72"/>
+      <c r="O6" s="72"/>
+      <c r="P6" s="72"/>
+      <c r="Q6" s="72"/>
+      <c r="S6" s="72" t="s">
         <v>15</v>
       </c>
-      <c r="T6" s="101"/>
-      <c r="U6" s="101"/>
-      <c r="V6" s="101"/>
-    </row>
-    <row r="8" spans="2:23" x14ac:dyDescent="0.3">
+      <c r="T6" s="72"/>
+      <c r="U6" s="72"/>
+      <c r="V6" s="72"/>
+    </row>
+    <row r="8" spans="2:23">
       <c r="B8" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="38" t="s">
+      <c r="C8" s="77" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="39"/>
-      <c r="E8" s="39"/>
-      <c r="F8" s="39"/>
-      <c r="G8" s="39"/>
-      <c r="H8" s="39"/>
-      <c r="I8" s="40"/>
+      <c r="D8" s="78"/>
+      <c r="E8" s="78"/>
+      <c r="F8" s="78"/>
+      <c r="G8" s="78"/>
+      <c r="H8" s="78"/>
+      <c r="I8" s="79"/>
       <c r="K8" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="S8" s="45" t="s">
+      <c r="S8" s="86" t="s">
         <v>19</v>
       </c>
-      <c r="T8" s="45"/>
-      <c r="U8" s="45"/>
+      <c r="T8" s="86"/>
+      <c r="U8" s="86"/>
       <c r="V8" s="28">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="2:23" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:23">
       <c r="B9" s="34" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="80" t="s">
+        <v>107</v>
+      </c>
+      <c r="D9" s="81"/>
+      <c r="E9" s="81"/>
+      <c r="F9" s="81"/>
+      <c r="G9" s="81"/>
+      <c r="H9" s="81"/>
+      <c r="I9" s="82"/>
+      <c r="K9" s="31"/>
+      <c r="S9" s="86" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="104" t="s">
-        <v>110</v>
-      </c>
-      <c r="D9" s="105"/>
-      <c r="E9" s="105"/>
-      <c r="F9" s="105"/>
-      <c r="G9" s="105"/>
-      <c r="H9" s="105"/>
-      <c r="I9" s="106"/>
-      <c r="K9" s="31"/>
-      <c r="S9" s="45" t="s">
-        <v>22</v>
-      </c>
-      <c r="T9" s="45"/>
-      <c r="U9" s="45"/>
+      <c r="T9" s="86"/>
+      <c r="U9" s="86"/>
       <c r="V9" s="28">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="2:23" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:23">
       <c r="B10" s="34" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="74" t="s">
+        <v>108</v>
+      </c>
+      <c r="D10" s="75"/>
+      <c r="E10" s="75"/>
+      <c r="F10" s="75"/>
+      <c r="G10" s="75"/>
+      <c r="H10" s="75"/>
+      <c r="I10" s="76"/>
+      <c r="K10" s="73" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="L10" s="73"/>
+      <c r="M10" s="73"/>
+      <c r="N10" s="73"/>
+      <c r="O10" s="73"/>
+      <c r="P10" s="73"/>
+      <c r="Q10" s="40"/>
+      <c r="R10" s="38"/>
+      <c r="S10" s="86" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="91" t="s">
-        <v>111</v>
-      </c>
-      <c r="D10" s="98"/>
-      <c r="E10" s="98"/>
-      <c r="F10" s="98"/>
-      <c r="G10" s="98"/>
-      <c r="H10" s="98"/>
-      <c r="I10" s="92"/>
-      <c r="K10" s="103" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
-      <c r="L10" s="103"/>
-      <c r="M10" s="103"/>
-      <c r="N10" s="103"/>
-      <c r="O10" s="103"/>
-      <c r="P10" s="103"/>
-      <c r="Q10" s="102"/>
-      <c r="R10" s="96"/>
-      <c r="S10" s="45" t="s">
+      <c r="T10" s="86" t="s">
         <v>24</v>
       </c>
-      <c r="T10" s="45" t="s">
-        <v>25</v>
-      </c>
-      <c r="U10" s="45"/>
+      <c r="U10" s="86"/>
       <c r="V10" s="28">
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="2:23" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:23">
       <c r="B11" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="74" t="s">
+        <v>109</v>
+      </c>
+      <c r="D11" s="75"/>
+      <c r="E11" s="75"/>
+      <c r="F11" s="75"/>
+      <c r="G11" s="75"/>
+      <c r="H11" s="75"/>
+      <c r="I11" s="76"/>
+      <c r="K11" s="73"/>
+      <c r="L11" s="73"/>
+      <c r="M11" s="73"/>
+      <c r="N11" s="73"/>
+      <c r="O11" s="73"/>
+      <c r="P11" s="73"/>
+      <c r="Q11" s="40"/>
+      <c r="R11" s="38"/>
+    </row>
+    <row r="12" spans="2:23">
+      <c r="B12" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="C12" s="74" t="s">
+        <v>98</v>
+      </c>
+      <c r="D12" s="75"/>
+      <c r="E12" s="75"/>
+      <c r="F12" s="75"/>
+      <c r="G12" s="75"/>
+      <c r="H12" s="75"/>
+      <c r="I12" s="76"/>
+      <c r="K12" s="73"/>
+      <c r="L12" s="73"/>
+      <c r="M12" s="73"/>
+      <c r="N12" s="73"/>
+      <c r="O12" s="73"/>
+      <c r="P12" s="73"/>
+      <c r="Q12" s="40"/>
+      <c r="R12" s="38"/>
+    </row>
+    <row r="13" spans="2:23">
+      <c r="B13" s="34" t="s">
+        <v>81</v>
+      </c>
+      <c r="C13" s="74" t="s">
+        <v>110</v>
+      </c>
+      <c r="D13" s="75"/>
+      <c r="E13" s="75"/>
+      <c r="F13" s="75"/>
+      <c r="G13" s="75"/>
+      <c r="H13" s="75"/>
+      <c r="I13" s="76"/>
+      <c r="K13" s="73"/>
+      <c r="L13" s="73"/>
+      <c r="M13" s="73"/>
+      <c r="N13" s="73"/>
+      <c r="O13" s="73"/>
+      <c r="P13" s="73"/>
+      <c r="Q13" s="68" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="91" t="s">
+      <c r="R13" s="69"/>
+      <c r="S13" s="69"/>
+      <c r="T13" s="69"/>
+      <c r="U13" s="69"/>
+      <c r="V13" s="69"/>
+      <c r="W13" s="69"/>
+    </row>
+    <row r="14" spans="2:23">
+      <c r="B14" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="C14" s="74" t="s">
+        <v>99</v>
+      </c>
+      <c r="D14" s="75"/>
+      <c r="E14" s="75"/>
+      <c r="F14" s="75"/>
+      <c r="G14" s="75"/>
+      <c r="H14" s="75"/>
+      <c r="I14" s="76"/>
+      <c r="K14" s="73"/>
+      <c r="L14" s="73"/>
+      <c r="M14" s="73"/>
+      <c r="N14" s="73"/>
+      <c r="O14" s="73"/>
+      <c r="P14" s="73"/>
+    </row>
+    <row r="15" spans="2:23">
+      <c r="B15" s="34" t="s">
+        <v>83</v>
+      </c>
+      <c r="C15" s="74" t="s">
         <v>112</v>
       </c>
-      <c r="D11" s="98"/>
-      <c r="E11" s="98"/>
-      <c r="F11" s="98"/>
-      <c r="G11" s="98"/>
-      <c r="H11" s="98"/>
-      <c r="I11" s="92"/>
-      <c r="K11" s="103"/>
-      <c r="L11" s="103"/>
-      <c r="M11" s="103"/>
-      <c r="N11" s="103"/>
-      <c r="O11" s="103"/>
-      <c r="P11" s="103"/>
-      <c r="Q11" s="102"/>
-      <c r="R11" s="96"/>
-    </row>
-    <row r="12" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B12" s="34" t="s">
-        <v>83</v>
-      </c>
-      <c r="C12" s="91" t="s">
+      <c r="D15" s="75"/>
+      <c r="E15" s="75"/>
+      <c r="F15" s="75"/>
+      <c r="G15" s="75"/>
+      <c r="H15" s="75"/>
+      <c r="I15" s="76"/>
+      <c r="K15" s="73"/>
+      <c r="L15" s="73"/>
+      <c r="M15" s="73"/>
+      <c r="N15" s="73"/>
+      <c r="O15" s="73"/>
+      <c r="P15" s="73"/>
+      <c r="Q15" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="R15" s="70" t="s">
+        <v>28</v>
+      </c>
+      <c r="S15" s="70"/>
+      <c r="T15" s="70"/>
+      <c r="U15" s="70"/>
+      <c r="V15" s="70"/>
+      <c r="W15" s="70"/>
+    </row>
+    <row r="16" spans="2:23">
+      <c r="B16" s="34" t="s">
+        <v>84</v>
+      </c>
+      <c r="C16" s="74" t="s">
+        <v>100</v>
+      </c>
+      <c r="D16" s="75"/>
+      <c r="E16" s="75"/>
+      <c r="F16" s="75"/>
+      <c r="G16" s="75"/>
+      <c r="H16" s="75"/>
+      <c r="I16" s="76"/>
+      <c r="K16" s="73"/>
+      <c r="L16" s="73"/>
+      <c r="M16" s="73"/>
+      <c r="N16" s="73"/>
+      <c r="O16" s="73"/>
+      <c r="P16" s="73"/>
+      <c r="Q16" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="R16" s="71" t="s">
+        <v>106</v>
+      </c>
+      <c r="S16" s="71"/>
+      <c r="T16" s="71"/>
+      <c r="U16" s="71"/>
+      <c r="V16" s="71"/>
+      <c r="W16" s="71"/>
+    </row>
+    <row r="17" spans="2:23">
+      <c r="B17" s="34" t="s">
+        <v>85</v>
+      </c>
+      <c r="C17" s="74" t="s">
         <v>101</v>
       </c>
-      <c r="D12" s="98"/>
-      <c r="E12" s="98"/>
-      <c r="F12" s="98"/>
-      <c r="G12" s="98"/>
-      <c r="H12" s="98"/>
-      <c r="I12" s="92"/>
-      <c r="K12" s="103"/>
-      <c r="L12" s="103"/>
-      <c r="M12" s="103"/>
-      <c r="N12" s="103"/>
-      <c r="O12" s="103"/>
-      <c r="P12" s="103"/>
-      <c r="Q12" s="102"/>
-      <c r="R12" s="96"/>
-    </row>
-    <row r="13" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B13" s="34" t="s">
-        <v>84</v>
-      </c>
-      <c r="C13" s="91" t="s">
+      <c r="D17" s="75"/>
+      <c r="E17" s="75"/>
+      <c r="F17" s="75"/>
+      <c r="G17" s="75"/>
+      <c r="H17" s="75"/>
+      <c r="I17" s="76"/>
+      <c r="K17" s="73"/>
+      <c r="L17" s="73"/>
+      <c r="M17" s="73"/>
+      <c r="N17" s="73"/>
+      <c r="O17" s="73"/>
+      <c r="P17" s="73"/>
+      <c r="Q17" s="29" t="s">
+        <v>30</v>
+      </c>
+      <c r="R17" s="71" t="s">
+        <v>119</v>
+      </c>
+      <c r="S17" s="71"/>
+      <c r="T17" s="71"/>
+      <c r="U17" s="71"/>
+      <c r="V17" s="71"/>
+      <c r="W17" s="71"/>
+    </row>
+    <row r="18" spans="2:23">
+      <c r="B18" s="34" t="s">
+        <v>86</v>
+      </c>
+      <c r="C18" s="74" t="s">
+        <v>102</v>
+      </c>
+      <c r="D18" s="75"/>
+      <c r="E18" s="75"/>
+      <c r="F18" s="75"/>
+      <c r="G18" s="75"/>
+      <c r="H18" s="75"/>
+      <c r="I18" s="76"/>
+      <c r="K18" s="73"/>
+      <c r="L18" s="73"/>
+      <c r="M18" s="73"/>
+      <c r="N18" s="73"/>
+      <c r="O18" s="73"/>
+      <c r="P18" s="73"/>
+      <c r="Q18" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="R18" s="71" t="s">
+        <v>122</v>
+      </c>
+      <c r="S18" s="71"/>
+      <c r="T18" s="71"/>
+      <c r="U18" s="71"/>
+      <c r="V18" s="71"/>
+      <c r="W18" s="71"/>
+    </row>
+    <row r="19" spans="2:23">
+      <c r="B19" s="34" t="s">
+        <v>87</v>
+      </c>
+      <c r="C19" s="74" t="s">
         <v>113</v>
       </c>
-      <c r="D13" s="98"/>
-      <c r="E13" s="98"/>
-      <c r="F13" s="98"/>
-      <c r="G13" s="98"/>
-      <c r="H13" s="98"/>
-      <c r="I13" s="92"/>
-      <c r="K13" s="103"/>
-      <c r="L13" s="103"/>
-      <c r="M13" s="103"/>
-      <c r="N13" s="103"/>
-      <c r="O13" s="103"/>
-      <c r="P13" s="103"/>
-      <c r="Q13" s="99" t="s">
-        <v>28</v>
-      </c>
-      <c r="R13" s="100"/>
-      <c r="S13" s="100"/>
-      <c r="T13" s="100"/>
-      <c r="U13" s="100"/>
-      <c r="V13" s="100"/>
-      <c r="W13" s="100"/>
-    </row>
-    <row r="14" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B14" s="34" t="s">
-        <v>85</v>
-      </c>
-      <c r="C14" s="91" t="s">
-        <v>102</v>
-      </c>
-      <c r="D14" s="98"/>
-      <c r="E14" s="98"/>
-      <c r="F14" s="98"/>
-      <c r="G14" s="98"/>
-      <c r="H14" s="98"/>
-      <c r="I14" s="92"/>
-      <c r="K14" s="103"/>
-      <c r="L14" s="103"/>
-      <c r="M14" s="103"/>
-      <c r="N14" s="103"/>
-      <c r="O14" s="103"/>
-      <c r="P14" s="103"/>
-    </row>
-    <row r="15" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B15" s="34" t="s">
-        <v>86</v>
-      </c>
-      <c r="C15" s="91" t="s">
+      <c r="D19" s="75"/>
+      <c r="E19" s="75"/>
+      <c r="F19" s="75"/>
+      <c r="G19" s="75"/>
+      <c r="H19" s="75"/>
+      <c r="I19" s="76"/>
+      <c r="K19" s="73"/>
+      <c r="L19" s="73"/>
+      <c r="M19" s="73"/>
+      <c r="N19" s="73"/>
+      <c r="O19" s="73"/>
+      <c r="P19" s="73"/>
+      <c r="Q19" s="29" t="s">
+        <v>120</v>
+      </c>
+      <c r="R19" s="71" t="s">
+        <v>151</v>
+      </c>
+      <c r="S19" s="71"/>
+      <c r="T19" s="71"/>
+      <c r="U19" s="71"/>
+      <c r="V19" s="71"/>
+      <c r="W19" s="71"/>
+    </row>
+    <row r="20" spans="2:23">
+      <c r="B20" s="34" t="s">
+        <v>88</v>
+      </c>
+      <c r="C20" s="74" t="s">
+        <v>114</v>
+      </c>
+      <c r="D20" s="75"/>
+      <c r="E20" s="75"/>
+      <c r="F20" s="75"/>
+      <c r="G20" s="75"/>
+      <c r="H20" s="75"/>
+      <c r="I20" s="76"/>
+      <c r="K20" s="73"/>
+      <c r="L20" s="73"/>
+      <c r="M20" s="73"/>
+      <c r="N20" s="73"/>
+      <c r="O20" s="73"/>
+      <c r="P20" s="73"/>
+      <c r="Q20" s="29" t="s">
+        <v>121</v>
+      </c>
+      <c r="R20" s="71" t="s">
+        <v>152</v>
+      </c>
+      <c r="S20" s="71"/>
+      <c r="T20" s="71"/>
+      <c r="U20" s="71"/>
+      <c r="V20" s="71"/>
+      <c r="W20" s="71"/>
+    </row>
+    <row r="21" spans="2:23">
+      <c r="B21" s="34" t="s">
+        <v>89</v>
+      </c>
+      <c r="C21" s="74" t="s">
         <v>115</v>
       </c>
-      <c r="D15" s="98"/>
-      <c r="E15" s="98"/>
-      <c r="F15" s="98"/>
-      <c r="G15" s="98"/>
-      <c r="H15" s="98"/>
-      <c r="I15" s="92"/>
-      <c r="K15" s="103"/>
-      <c r="L15" s="103"/>
-      <c r="M15" s="103"/>
-      <c r="N15" s="103"/>
-      <c r="O15" s="103"/>
-      <c r="P15" s="103"/>
-      <c r="Q15" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="R15" s="46" t="s">
-        <v>30</v>
-      </c>
-      <c r="S15" s="46"/>
-      <c r="T15" s="46"/>
-      <c r="U15" s="46"/>
-      <c r="V15" s="46"/>
-      <c r="W15" s="46"/>
-    </row>
-    <row r="16" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B16" s="34" t="s">
-        <v>87</v>
-      </c>
-      <c r="C16" s="91" t="s">
+      <c r="D21" s="75"/>
+      <c r="E21" s="75"/>
+      <c r="F21" s="75"/>
+      <c r="G21" s="75"/>
+      <c r="H21" s="75"/>
+      <c r="I21" s="76"/>
+      <c r="K21" s="73"/>
+      <c r="L21" s="73"/>
+      <c r="M21" s="73"/>
+      <c r="N21" s="73"/>
+      <c r="O21" s="73"/>
+      <c r="P21" s="73"/>
+      <c r="Q21" s="40"/>
+      <c r="R21" s="38"/>
+      <c r="S21" s="39"/>
+    </row>
+    <row r="22" spans="2:23">
+      <c r="B22" s="34" t="s">
+        <v>90</v>
+      </c>
+      <c r="C22" s="74" t="s">
+        <v>116</v>
+      </c>
+      <c r="D22" s="75"/>
+      <c r="E22" s="75"/>
+      <c r="F22" s="75"/>
+      <c r="G22" s="75"/>
+      <c r="H22" s="75"/>
+      <c r="I22" s="76"/>
+      <c r="K22" s="73"/>
+      <c r="L22" s="73"/>
+      <c r="M22" s="73"/>
+      <c r="N22" s="73"/>
+      <c r="O22" s="73"/>
+      <c r="P22" s="73"/>
+      <c r="Q22" s="40"/>
+    </row>
+    <row r="23" spans="2:23">
+      <c r="B23" s="34" t="s">
+        <v>91</v>
+      </c>
+      <c r="C23" s="74" t="s">
         <v>103</v>
       </c>
-      <c r="D16" s="98"/>
-      <c r="E16" s="98"/>
-      <c r="F16" s="98"/>
-      <c r="G16" s="98"/>
-      <c r="H16" s="98"/>
-      <c r="I16" s="92"/>
-      <c r="K16" s="103"/>
-      <c r="L16" s="103"/>
-      <c r="M16" s="103"/>
-      <c r="N16" s="103"/>
-      <c r="O16" s="103"/>
-      <c r="P16" s="103"/>
-      <c r="Q16" s="29" t="s">
-        <v>31</v>
-      </c>
-      <c r="R16" s="41" t="s">
-        <v>109</v>
-      </c>
-      <c r="S16" s="41"/>
-      <c r="T16" s="41"/>
-      <c r="U16" s="41"/>
-      <c r="V16" s="41"/>
-      <c r="W16" s="41"/>
-    </row>
-    <row r="17" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B17" s="34" t="s">
-        <v>88</v>
-      </c>
-      <c r="C17" s="91" t="s">
+      <c r="D23" s="75"/>
+      <c r="E23" s="75"/>
+      <c r="F23" s="75"/>
+      <c r="G23" s="75"/>
+      <c r="H23" s="75"/>
+      <c r="I23" s="76"/>
+      <c r="K23" s="73"/>
+      <c r="L23" s="73"/>
+      <c r="M23" s="73"/>
+      <c r="N23" s="73"/>
+      <c r="O23" s="73"/>
+      <c r="P23" s="73"/>
+      <c r="Q23" s="40"/>
+    </row>
+    <row r="24" spans="2:23">
+      <c r="B24" s="34" t="s">
+        <v>92</v>
+      </c>
+      <c r="C24" s="74" t="s">
         <v>104</v>
       </c>
-      <c r="D17" s="98"/>
-      <c r="E17" s="98"/>
-      <c r="F17" s="98"/>
-      <c r="G17" s="98"/>
-      <c r="H17" s="98"/>
-      <c r="I17" s="92"/>
-      <c r="K17" s="103"/>
-      <c r="L17" s="103"/>
-      <c r="M17" s="103"/>
-      <c r="N17" s="103"/>
-      <c r="O17" s="103"/>
-      <c r="P17" s="103"/>
-      <c r="Q17" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="R17" s="41" t="s">
-        <v>122</v>
-      </c>
-      <c r="S17" s="41"/>
-      <c r="T17" s="41"/>
-      <c r="U17" s="41"/>
-      <c r="V17" s="41"/>
-      <c r="W17" s="41"/>
-    </row>
-    <row r="18" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B18" s="34" t="s">
-        <v>89</v>
-      </c>
-      <c r="C18" s="91" t="s">
+      <c r="D24" s="75"/>
+      <c r="E24" s="75"/>
+      <c r="F24" s="75"/>
+      <c r="G24" s="75"/>
+      <c r="H24" s="75"/>
+      <c r="I24" s="76"/>
+      <c r="K24" s="73"/>
+      <c r="L24" s="73"/>
+      <c r="M24" s="73"/>
+      <c r="N24" s="73"/>
+      <c r="O24" s="73"/>
+      <c r="P24" s="73"/>
+      <c r="Q24" s="40"/>
+    </row>
+    <row r="25" spans="2:23">
+      <c r="B25" s="34" t="s">
+        <v>93</v>
+      </c>
+      <c r="C25" s="74" t="s">
+        <v>117</v>
+      </c>
+      <c r="D25" s="75"/>
+      <c r="E25" s="75"/>
+      <c r="F25" s="75"/>
+      <c r="G25" s="75"/>
+      <c r="H25" s="75"/>
+      <c r="I25" s="76"/>
+      <c r="K25" s="73"/>
+      <c r="L25" s="73"/>
+      <c r="M25" s="73"/>
+      <c r="N25" s="73"/>
+      <c r="O25" s="73"/>
+      <c r="P25" s="73"/>
+    </row>
+    <row r="26" spans="2:23">
+      <c r="B26" s="34" t="s">
+        <v>94</v>
+      </c>
+      <c r="C26" s="74" t="s">
+        <v>118</v>
+      </c>
+      <c r="D26" s="75"/>
+      <c r="E26" s="75"/>
+      <c r="F26" s="75"/>
+      <c r="G26" s="75"/>
+      <c r="H26" s="75"/>
+      <c r="I26" s="76"/>
+      <c r="K26" s="73"/>
+      <c r="L26" s="73"/>
+      <c r="M26" s="73"/>
+      <c r="N26" s="73"/>
+      <c r="O26" s="73"/>
+      <c r="P26" s="73"/>
+    </row>
+    <row r="27" spans="2:23">
+      <c r="B27" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="C27" s="74" t="s">
         <v>105</v>
       </c>
-      <c r="D18" s="98"/>
-      <c r="E18" s="98"/>
-      <c r="F18" s="98"/>
-      <c r="G18" s="98"/>
-      <c r="H18" s="98"/>
-      <c r="I18" s="92"/>
-      <c r="K18" s="103"/>
-      <c r="L18" s="103"/>
-      <c r="M18" s="103"/>
-      <c r="N18" s="103"/>
-      <c r="O18" s="103"/>
-      <c r="P18" s="103"/>
-      <c r="Q18" s="29" t="s">
-        <v>33</v>
-      </c>
-      <c r="R18" s="41" t="s">
-        <v>125</v>
-      </c>
-      <c r="S18" s="41"/>
-      <c r="T18" s="41"/>
-      <c r="U18" s="41"/>
-      <c r="V18" s="41"/>
-      <c r="W18" s="41"/>
-    </row>
-    <row r="19" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B19" s="34" t="s">
-        <v>90</v>
-      </c>
-      <c r="C19" s="91" t="s">
-        <v>116</v>
-      </c>
-      <c r="D19" s="98"/>
-      <c r="E19" s="98"/>
-      <c r="F19" s="98"/>
-      <c r="G19" s="98"/>
-      <c r="H19" s="98"/>
-      <c r="I19" s="92"/>
-      <c r="K19" s="103"/>
-      <c r="L19" s="103"/>
-      <c r="M19" s="103"/>
-      <c r="N19" s="103"/>
-      <c r="O19" s="103"/>
-      <c r="P19" s="103"/>
-      <c r="Q19" s="29" t="s">
-        <v>123</v>
-      </c>
-      <c r="R19" s="41" t="s">
-        <v>159</v>
-      </c>
-      <c r="S19" s="41"/>
-      <c r="T19" s="41"/>
-      <c r="U19" s="41"/>
-      <c r="V19" s="41"/>
-      <c r="W19" s="41"/>
-    </row>
-    <row r="20" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B20" s="34" t="s">
-        <v>91</v>
-      </c>
-      <c r="C20" s="91" t="s">
-        <v>117</v>
-      </c>
-      <c r="D20" s="98"/>
-      <c r="E20" s="98"/>
-      <c r="F20" s="98"/>
-      <c r="G20" s="98"/>
-      <c r="H20" s="98"/>
-      <c r="I20" s="92"/>
-      <c r="K20" s="103"/>
-      <c r="L20" s="103"/>
-      <c r="M20" s="103"/>
-      <c r="N20" s="103"/>
-      <c r="O20" s="103"/>
-      <c r="P20" s="103"/>
-      <c r="Q20" s="29" t="s">
-        <v>124</v>
-      </c>
-      <c r="R20" s="41" t="s">
-        <v>160</v>
-      </c>
-      <c r="S20" s="41"/>
-      <c r="T20" s="41"/>
-      <c r="U20" s="41"/>
-      <c r="V20" s="41"/>
-      <c r="W20" s="41"/>
-    </row>
-    <row r="21" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B21" s="34" t="s">
-        <v>92</v>
-      </c>
-      <c r="C21" s="91" t="s">
-        <v>118</v>
-      </c>
-      <c r="D21" s="98"/>
-      <c r="E21" s="98"/>
-      <c r="F21" s="98"/>
-      <c r="G21" s="98"/>
-      <c r="H21" s="98"/>
-      <c r="I21" s="92"/>
-      <c r="K21" s="103"/>
-      <c r="L21" s="103"/>
-      <c r="M21" s="103"/>
-      <c r="N21" s="103"/>
-      <c r="O21" s="103"/>
-      <c r="P21" s="103"/>
-      <c r="Q21" s="102"/>
-      <c r="R21" s="96"/>
-      <c r="S21" s="97"/>
-      <c r="T21" s="107"/>
-      <c r="U21" s="107"/>
-      <c r="V21" s="107"/>
-    </row>
-    <row r="22" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B22" s="34" t="s">
-        <v>93</v>
-      </c>
-      <c r="C22" s="91" t="s">
-        <v>119</v>
-      </c>
-      <c r="D22" s="98"/>
-      <c r="E22" s="98"/>
-      <c r="F22" s="98"/>
-      <c r="G22" s="98"/>
-      <c r="H22" s="98"/>
-      <c r="I22" s="92"/>
-      <c r="K22" s="103"/>
-      <c r="L22" s="103"/>
-      <c r="M22" s="103"/>
-      <c r="N22" s="103"/>
-      <c r="O22" s="103"/>
-      <c r="P22" s="103"/>
-      <c r="Q22" s="102"/>
-    </row>
-    <row r="23" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B23" s="34" t="s">
-        <v>94</v>
-      </c>
-      <c r="C23" s="91" t="s">
-        <v>106</v>
-      </c>
-      <c r="D23" s="98"/>
-      <c r="E23" s="98"/>
-      <c r="F23" s="98"/>
-      <c r="G23" s="98"/>
-      <c r="H23" s="98"/>
-      <c r="I23" s="92"/>
-      <c r="K23" s="103"/>
-      <c r="L23" s="103"/>
-      <c r="M23" s="103"/>
-      <c r="N23" s="103"/>
-      <c r="O23" s="103"/>
-      <c r="P23" s="103"/>
-      <c r="Q23" s="102"/>
-    </row>
-    <row r="24" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B24" s="34" t="s">
-        <v>95</v>
-      </c>
-      <c r="C24" s="91" t="s">
-        <v>107</v>
-      </c>
-      <c r="D24" s="98"/>
-      <c r="E24" s="98"/>
-      <c r="F24" s="98"/>
-      <c r="G24" s="98"/>
-      <c r="H24" s="98"/>
-      <c r="I24" s="92"/>
-      <c r="K24" s="103"/>
-      <c r="L24" s="103"/>
-      <c r="M24" s="103"/>
-      <c r="N24" s="103"/>
-      <c r="O24" s="103"/>
-      <c r="P24" s="103"/>
-      <c r="Q24" s="102"/>
-    </row>
-    <row r="25" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B25" s="34" t="s">
+      <c r="D27" s="75"/>
+      <c r="E27" s="75"/>
+      <c r="F27" s="75"/>
+      <c r="G27" s="75"/>
+      <c r="H27" s="75"/>
+      <c r="I27" s="76"/>
+      <c r="K27" s="73"/>
+      <c r="L27" s="73"/>
+      <c r="M27" s="73"/>
+      <c r="N27" s="73"/>
+      <c r="O27" s="73"/>
+      <c r="P27" s="73"/>
+    </row>
+    <row r="28" spans="2:23">
+      <c r="B28" s="34" t="s">
         <v>96</v>
       </c>
-      <c r="C25" s="91" t="s">
-        <v>120</v>
-      </c>
-      <c r="D25" s="98"/>
-      <c r="E25" s="98"/>
-      <c r="F25" s="98"/>
-      <c r="G25" s="98"/>
-      <c r="H25" s="98"/>
-      <c r="I25" s="92"/>
-      <c r="K25" s="103"/>
-      <c r="L25" s="103"/>
-      <c r="M25" s="103"/>
-      <c r="N25" s="103"/>
-      <c r="O25" s="103"/>
-      <c r="P25" s="103"/>
-    </row>
-    <row r="26" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B26" s="34" t="s">
+      <c r="C28" s="74" t="s">
+        <v>98</v>
+      </c>
+      <c r="D28" s="75"/>
+      <c r="E28" s="75"/>
+      <c r="F28" s="75"/>
+      <c r="G28" s="75"/>
+      <c r="H28" s="75"/>
+      <c r="I28" s="76"/>
+      <c r="K28" s="73"/>
+      <c r="L28" s="73"/>
+      <c r="M28" s="73"/>
+      <c r="N28" s="73"/>
+      <c r="O28" s="73"/>
+      <c r="P28" s="73"/>
+    </row>
+    <row r="29" spans="2:23">
+      <c r="B29" s="34" t="s">
         <v>97</v>
       </c>
-      <c r="C26" s="91" t="s">
-        <v>121</v>
-      </c>
-      <c r="D26" s="98"/>
-      <c r="E26" s="98"/>
-      <c r="F26" s="98"/>
-      <c r="G26" s="98"/>
-      <c r="H26" s="98"/>
-      <c r="I26" s="92"/>
-      <c r="K26" s="103"/>
-      <c r="L26" s="103"/>
-      <c r="M26" s="103"/>
-      <c r="N26" s="103"/>
-      <c r="O26" s="103"/>
-      <c r="P26" s="103"/>
-    </row>
-    <row r="27" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B27" s="34" t="s">
-        <v>98</v>
-      </c>
-      <c r="C27" s="91" t="s">
-        <v>108</v>
-      </c>
-      <c r="D27" s="98"/>
-      <c r="E27" s="98"/>
-      <c r="F27" s="98"/>
-      <c r="G27" s="98"/>
-      <c r="H27" s="98"/>
-      <c r="I27" s="92"/>
-      <c r="K27" s="103"/>
-      <c r="L27" s="103"/>
-      <c r="M27" s="103"/>
-      <c r="N27" s="103"/>
-      <c r="O27" s="103"/>
-      <c r="P27" s="103"/>
-    </row>
-    <row r="28" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B28" s="34" t="s">
-        <v>99</v>
-      </c>
-      <c r="C28" s="91" t="s">
-        <v>101</v>
-      </c>
-      <c r="D28" s="98"/>
-      <c r="E28" s="98"/>
-      <c r="F28" s="98"/>
-      <c r="G28" s="98"/>
-      <c r="H28" s="98"/>
-      <c r="I28" s="92"/>
-      <c r="K28" s="103"/>
-      <c r="L28" s="103"/>
-      <c r="M28" s="103"/>
-      <c r="N28" s="103"/>
-      <c r="O28" s="103"/>
-      <c r="P28" s="103"/>
-    </row>
-    <row r="29" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B29" s="34" t="s">
-        <v>100</v>
-      </c>
-      <c r="C29" s="93" t="s">
-        <v>114</v>
-      </c>
-      <c r="D29" s="94"/>
-      <c r="E29" s="94"/>
-      <c r="F29" s="94"/>
-      <c r="G29" s="94"/>
-      <c r="H29" s="94"/>
-      <c r="I29" s="95"/>
-      <c r="K29" s="103"/>
-      <c r="L29" s="103"/>
-      <c r="M29" s="103"/>
-      <c r="N29" s="103"/>
-      <c r="O29" s="103"/>
-      <c r="P29" s="103"/>
-    </row>
-    <row r="30" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="K30" s="103"/>
-      <c r="L30" s="103"/>
-      <c r="M30" s="103"/>
-      <c r="N30" s="103"/>
-      <c r="O30" s="103"/>
-      <c r="P30" s="103"/>
-    </row>
-    <row r="31" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="K31" s="103"/>
-      <c r="L31" s="103"/>
-      <c r="M31" s="103"/>
-      <c r="N31" s="103"/>
-      <c r="O31" s="103"/>
-      <c r="P31" s="103"/>
-    </row>
-    <row r="32" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="K32" s="103"/>
-      <c r="L32" s="103"/>
-      <c r="M32" s="103"/>
-      <c r="N32" s="103"/>
-      <c r="O32" s="103"/>
-      <c r="P32" s="103"/>
+      <c r="C29" s="87" t="s">
+        <v>111</v>
+      </c>
+      <c r="D29" s="88"/>
+      <c r="E29" s="88"/>
+      <c r="F29" s="88"/>
+      <c r="G29" s="88"/>
+      <c r="H29" s="88"/>
+      <c r="I29" s="89"/>
+      <c r="K29" s="73"/>
+      <c r="L29" s="73"/>
+      <c r="M29" s="73"/>
+      <c r="N29" s="73"/>
+      <c r="O29" s="73"/>
+      <c r="P29" s="73"/>
+    </row>
+    <row r="30" spans="2:23">
+      <c r="K30" s="73"/>
+      <c r="L30" s="73"/>
+      <c r="M30" s="73"/>
+      <c r="N30" s="73"/>
+      <c r="O30" s="73"/>
+      <c r="P30" s="73"/>
+    </row>
+    <row r="31" spans="2:23">
+      <c r="K31" s="73"/>
+      <c r="L31" s="73"/>
+      <c r="M31" s="73"/>
+      <c r="N31" s="73"/>
+      <c r="O31" s="73"/>
+      <c r="P31" s="73"/>
+    </row>
+    <row r="32" spans="2:23">
+      <c r="K32" s="73"/>
+      <c r="L32" s="73"/>
+      <c r="M32" s="73"/>
+      <c r="N32" s="73"/>
+      <c r="O32" s="73"/>
+      <c r="P32" s="73"/>
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="Q13:W13"/>
-    <mergeCell ref="R15:W15"/>
-    <mergeCell ref="R16:W16"/>
-    <mergeCell ref="R17:W17"/>
-    <mergeCell ref="R18:W18"/>
+    <mergeCell ref="C25:I25"/>
+    <mergeCell ref="C26:I26"/>
+    <mergeCell ref="C27:I27"/>
+    <mergeCell ref="C28:I28"/>
+    <mergeCell ref="C29:I29"/>
+    <mergeCell ref="D1:I1"/>
+    <mergeCell ref="B3:K3"/>
+    <mergeCell ref="S10:U10"/>
+    <mergeCell ref="S8:U8"/>
+    <mergeCell ref="K6:Q6"/>
+    <mergeCell ref="S6:V6"/>
+    <mergeCell ref="S9:U9"/>
+    <mergeCell ref="C15:I15"/>
+    <mergeCell ref="C16:I16"/>
+    <mergeCell ref="C17:I17"/>
+    <mergeCell ref="C18:I18"/>
+    <mergeCell ref="C19:I19"/>
     <mergeCell ref="R19:W19"/>
     <mergeCell ref="R20:W20"/>
     <mergeCell ref="B6:I6"/>
@@ -3655,23 +3734,11 @@
     <mergeCell ref="C12:I12"/>
     <mergeCell ref="C13:I13"/>
     <mergeCell ref="C14:I14"/>
-    <mergeCell ref="C15:I15"/>
-    <mergeCell ref="C16:I16"/>
-    <mergeCell ref="C17:I17"/>
-    <mergeCell ref="C18:I18"/>
-    <mergeCell ref="C19:I19"/>
-    <mergeCell ref="D1:I1"/>
-    <mergeCell ref="B3:K3"/>
-    <mergeCell ref="S10:U10"/>
-    <mergeCell ref="S8:U8"/>
-    <mergeCell ref="K6:Q6"/>
-    <mergeCell ref="S6:V6"/>
-    <mergeCell ref="S9:U9"/>
-    <mergeCell ref="C25:I25"/>
-    <mergeCell ref="C26:I26"/>
-    <mergeCell ref="C27:I27"/>
-    <mergeCell ref="C28:I28"/>
-    <mergeCell ref="C29:I29"/>
+    <mergeCell ref="Q13:W13"/>
+    <mergeCell ref="R15:W15"/>
+    <mergeCell ref="R16:W16"/>
+    <mergeCell ref="R17:W17"/>
+    <mergeCell ref="R18:W18"/>
   </mergeCells>
   <phoneticPr fontId="17" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3685,7 +3752,7 @@
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="B1:AB15"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="12.33203125" customWidth="1"/>
     <col min="3" max="3" width="17.33203125" customWidth="1"/>
@@ -3706,239 +3773,239 @@
     <col min="28" max="28" width="5.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:28" ht="15" thickBot="1">
       <c r="B1" s="11"/>
-      <c r="D1" s="152" t="s">
+      <c r="D1" s="126" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="153"/>
-      <c r="F1" s="153"/>
-      <c r="G1" s="154"/>
-    </row>
-    <row r="2" spans="2:28" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="3" spans="2:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="149" t="s">
+      <c r="E1" s="127"/>
+      <c r="F1" s="127"/>
+      <c r="G1" s="128"/>
+    </row>
+    <row r="2" spans="2:28" ht="15" thickBot="1"/>
+    <row r="3" spans="2:28" ht="15" thickBot="1">
+      <c r="B3" s="95" t="s">
+        <v>123</v>
+      </c>
+      <c r="C3" s="96"/>
+      <c r="D3" s="96"/>
+      <c r="E3" s="96"/>
+      <c r="F3" s="96"/>
+      <c r="G3" s="97"/>
+    </row>
+    <row r="4" spans="2:28" ht="15" thickBot="1"/>
+    <row r="5" spans="2:28" ht="15.6">
+      <c r="B5" s="129" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" s="103" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="104"/>
+      <c r="E5" s="105"/>
+      <c r="F5" s="109" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" s="110"/>
+      <c r="H5" s="93" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" s="93"/>
+      <c r="J5" s="93"/>
+      <c r="K5" s="93"/>
+      <c r="L5" s="93"/>
+      <c r="M5" s="93"/>
+      <c r="N5" s="93"/>
+      <c r="O5" s="93"/>
+      <c r="P5" s="93"/>
+      <c r="Q5" s="93"/>
+      <c r="R5" s="93"/>
+      <c r="S5" s="93"/>
+      <c r="T5" s="93"/>
+      <c r="U5" s="93"/>
+      <c r="V5" s="93"/>
+      <c r="W5" s="93"/>
+      <c r="X5" s="93"/>
+      <c r="Y5" s="93"/>
+      <c r="Z5" s="93"/>
+      <c r="AA5" s="93"/>
+      <c r="AB5" s="94"/>
+    </row>
+    <row r="6" spans="2:28" ht="15.6" customHeight="1">
+      <c r="B6" s="130"/>
+      <c r="C6" s="106"/>
+      <c r="D6" s="107"/>
+      <c r="E6" s="108"/>
+      <c r="F6" s="111"/>
+      <c r="G6" s="112"/>
+      <c r="H6" s="100" t="s">
+        <v>36</v>
+      </c>
+      <c r="I6" s="119" t="s">
+        <v>37</v>
+      </c>
+      <c r="J6" s="120"/>
+      <c r="K6" s="120"/>
+      <c r="L6" s="120"/>
+      <c r="M6" s="120"/>
+      <c r="N6" s="120"/>
+      <c r="O6" s="120"/>
+      <c r="P6" s="121"/>
+      <c r="Q6" s="90" t="s">
+        <v>38</v>
+      </c>
+      <c r="R6" s="91"/>
+      <c r="S6" s="91"/>
+      <c r="T6" s="91"/>
+      <c r="U6" s="92"/>
+      <c r="V6" s="124" t="s">
+        <v>39</v>
+      </c>
+      <c r="W6" s="124"/>
+      <c r="X6" s="124"/>
+      <c r="Y6" s="124"/>
+      <c r="Z6" s="124"/>
+      <c r="AA6" s="124"/>
+      <c r="AB6" s="122"/>
+    </row>
+    <row r="7" spans="2:28" ht="15.6">
+      <c r="B7" s="130"/>
+      <c r="C7" s="98" t="s">
+        <v>124</v>
+      </c>
+      <c r="D7" s="113" t="s">
+        <v>125</v>
+      </c>
+      <c r="E7" s="115" t="s">
+        <v>126</v>
+      </c>
+      <c r="F7" s="117" t="s">
+        <v>127</v>
+      </c>
+      <c r="G7" s="115" t="s">
+        <v>133</v>
+      </c>
+      <c r="H7" s="101"/>
+      <c r="I7" s="123" t="s">
+        <v>128</v>
+      </c>
+      <c r="J7" s="123"/>
+      <c r="K7" s="123" t="s">
+        <v>129</v>
+      </c>
+      <c r="L7" s="123"/>
+      <c r="M7" s="123" t="s">
         <v>130</v>
       </c>
-      <c r="C3" s="150"/>
-      <c r="D3" s="150"/>
-      <c r="E3" s="150"/>
-      <c r="F3" s="150"/>
-      <c r="G3" s="151"/>
-    </row>
-    <row r="4" spans="2:28" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="5" spans="2:28" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B5" s="138" t="s">
-        <v>34</v>
-      </c>
-      <c r="C5" s="142" t="s">
-        <v>35</v>
-      </c>
-      <c r="D5" s="118"/>
-      <c r="E5" s="143"/>
-      <c r="F5" s="163" t="s">
-        <v>36</v>
-      </c>
-      <c r="G5" s="130"/>
-      <c r="H5" s="119" t="s">
-        <v>37</v>
-      </c>
-      <c r="I5" s="119"/>
-      <c r="J5" s="119"/>
-      <c r="K5" s="119"/>
-      <c r="L5" s="119"/>
-      <c r="M5" s="119"/>
-      <c r="N5" s="119"/>
-      <c r="O5" s="119"/>
-      <c r="P5" s="119"/>
-      <c r="Q5" s="119"/>
-      <c r="R5" s="119"/>
-      <c r="S5" s="119"/>
-      <c r="T5" s="119"/>
-      <c r="U5" s="119"/>
-      <c r="V5" s="119"/>
-      <c r="W5" s="119"/>
-      <c r="X5" s="119"/>
-      <c r="Y5" s="119"/>
-      <c r="Z5" s="119"/>
-      <c r="AA5" s="119"/>
-      <c r="AB5" s="120"/>
-    </row>
-    <row r="6" spans="2:28" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="139"/>
-      <c r="C6" s="144"/>
-      <c r="D6" s="110"/>
-      <c r="E6" s="145"/>
-      <c r="F6" s="117"/>
-      <c r="G6" s="131"/>
-      <c r="H6" s="125" t="s">
-        <v>38</v>
-      </c>
-      <c r="I6" s="111" t="s">
-        <v>39</v>
-      </c>
-      <c r="J6" s="112"/>
-      <c r="K6" s="112"/>
-      <c r="L6" s="112"/>
-      <c r="M6" s="112"/>
-      <c r="N6" s="112"/>
-      <c r="O6" s="112"/>
-      <c r="P6" s="113"/>
-      <c r="Q6" s="114" t="s">
+      <c r="N7" s="123"/>
+      <c r="O7" s="123" t="s">
+        <v>131</v>
+      </c>
+      <c r="P7" s="123"/>
+      <c r="Q7" s="125" t="s">
+        <v>29</v>
+      </c>
+      <c r="R7" s="125" t="s">
+        <v>30</v>
+      </c>
+      <c r="S7" s="125" t="s">
+        <v>31</v>
+      </c>
+      <c r="T7" s="125" t="s">
+        <v>120</v>
+      </c>
+      <c r="U7" s="125" t="s">
+        <v>121</v>
+      </c>
+      <c r="V7" s="124">
+        <v>0</v>
+      </c>
+      <c r="W7" s="124">
+        <v>1</v>
+      </c>
+      <c r="X7" s="124">
+        <v>2</v>
+      </c>
+      <c r="Y7" s="124" t="s">
         <v>40</v>
       </c>
-      <c r="R6" s="115"/>
-      <c r="S6" s="115"/>
-      <c r="T6" s="115"/>
-      <c r="U6" s="116"/>
-      <c r="V6" s="49" t="s">
+      <c r="Z7" s="124" t="s">
         <v>41</v>
       </c>
-      <c r="W6" s="49"/>
-      <c r="X6" s="49"/>
-      <c r="Y6" s="49"/>
-      <c r="Z6" s="49"/>
-      <c r="AA6" s="49"/>
-      <c r="AB6" s="121"/>
-    </row>
-    <row r="7" spans="2:28" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B7" s="139"/>
-      <c r="C7" s="132" t="s">
-        <v>131</v>
-      </c>
-      <c r="D7" s="47" t="s">
+      <c r="AA7" s="124" t="s">
+        <v>42</v>
+      </c>
+      <c r="AB7" s="122" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="2:28" ht="15.6" customHeight="1">
+      <c r="B8" s="130"/>
+      <c r="C8" s="99"/>
+      <c r="D8" s="114"/>
+      <c r="E8" s="116"/>
+      <c r="F8" s="118"/>
+      <c r="G8" s="116"/>
+      <c r="H8" s="102"/>
+      <c r="I8" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="J8" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="K8" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="L8" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="M8" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="N8" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="O8" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="P8" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q8" s="125"/>
+      <c r="R8" s="125"/>
+      <c r="S8" s="125"/>
+      <c r="T8" s="125"/>
+      <c r="U8" s="125"/>
+      <c r="V8" s="124"/>
+      <c r="W8" s="124"/>
+      <c r="X8" s="124"/>
+      <c r="Y8" s="124"/>
+      <c r="Z8" s="124"/>
+      <c r="AA8" s="124"/>
+      <c r="AB8" s="122"/>
+    </row>
+    <row r="9" spans="2:28" ht="15.6">
+      <c r="B9" s="48" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" s="51">
+        <v>1</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="E9" s="50" t="s">
         <v>132</v>
       </c>
-      <c r="E7" s="133" t="s">
-        <v>133</v>
-      </c>
-      <c r="F7" s="108" t="s">
+      <c r="F9" t="s">
         <v>134</v>
       </c>
-      <c r="G7" s="133" t="s">
-        <v>140</v>
-      </c>
-      <c r="H7" s="126"/>
-      <c r="I7" s="51" t="s">
+      <c r="G9" s="46"/>
+      <c r="H9" s="44" t="s">
         <v>135</v>
       </c>
-      <c r="J7" s="51"/>
-      <c r="K7" s="51" t="s">
+      <c r="I9" s="14" t="s">
         <v>136</v>
-      </c>
-      <c r="L7" s="51"/>
-      <c r="M7" s="51" t="s">
-        <v>137</v>
-      </c>
-      <c r="N7" s="51"/>
-      <c r="O7" s="51" t="s">
-        <v>138</v>
-      </c>
-      <c r="P7" s="51"/>
-      <c r="Q7" s="50" t="s">
-        <v>31</v>
-      </c>
-      <c r="R7" s="50" t="s">
-        <v>32</v>
-      </c>
-      <c r="S7" s="50" t="s">
-        <v>33</v>
-      </c>
-      <c r="T7" s="50" t="s">
-        <v>123</v>
-      </c>
-      <c r="U7" s="50" t="s">
-        <v>124</v>
-      </c>
-      <c r="V7" s="49">
-        <v>0</v>
-      </c>
-      <c r="W7" s="49">
-        <v>1</v>
-      </c>
-      <c r="X7" s="49">
-        <v>2</v>
-      </c>
-      <c r="Y7" s="49" t="s">
-        <v>42</v>
-      </c>
-      <c r="Z7" s="49" t="s">
-        <v>43</v>
-      </c>
-      <c r="AA7" s="49" t="s">
-        <v>44</v>
-      </c>
-      <c r="AB7" s="121" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="8" spans="2:28" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="139"/>
-      <c r="C8" s="134"/>
-      <c r="D8" s="48"/>
-      <c r="E8" s="135"/>
-      <c r="F8" s="109"/>
-      <c r="G8" s="135"/>
-      <c r="H8" s="127"/>
-      <c r="I8" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="J8" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="K8" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="L8" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="M8" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="N8" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="O8" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="P8" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q8" s="50"/>
-      <c r="R8" s="50"/>
-      <c r="S8" s="50"/>
-      <c r="T8" s="50"/>
-      <c r="U8" s="50"/>
-      <c r="V8" s="49"/>
-      <c r="W8" s="49"/>
-      <c r="X8" s="49"/>
-      <c r="Y8" s="49"/>
-      <c r="Z8" s="49"/>
-      <c r="AA8" s="49"/>
-      <c r="AB8" s="121"/>
-    </row>
-    <row r="9" spans="2:28" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B9" s="140" t="s">
-        <v>48</v>
-      </c>
-      <c r="C9" s="147">
-        <v>1</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>145</v>
-      </c>
-      <c r="E9" s="146" t="s">
-        <v>139</v>
-      </c>
-      <c r="F9" t="s">
-        <v>141</v>
-      </c>
-      <c r="G9" s="136"/>
-      <c r="H9" s="128" t="s">
-        <v>142</v>
-      </c>
-      <c r="I9" s="14" t="s">
-        <v>143</v>
       </c>
       <c r="J9" s="14"/>
       <c r="K9" s="14"/>
@@ -3948,51 +4015,51 @@
       <c r="O9" s="14"/>
       <c r="P9" s="14"/>
       <c r="Q9" s="15" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="R9" s="15"/>
       <c r="S9" s="15"/>
       <c r="T9" s="15"/>
       <c r="U9" s="15"/>
-      <c r="V9" s="155" t="s">
-        <v>143</v>
-      </c>
-      <c r="W9" s="155"/>
-      <c r="X9" s="155"/>
-      <c r="Y9" s="155"/>
-      <c r="Z9" s="155"/>
-      <c r="AA9" s="155"/>
-      <c r="AB9" s="156"/>
-    </row>
-    <row r="10" spans="2:28" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B10" s="140" t="s">
-        <v>49</v>
-      </c>
-      <c r="C10" s="147">
+      <c r="V9" s="53" t="s">
+        <v>136</v>
+      </c>
+      <c r="W9" s="53"/>
+      <c r="X9" s="53"/>
+      <c r="Y9" s="53"/>
+      <c r="Z9" s="53"/>
+      <c r="AA9" s="53"/>
+      <c r="AB9" s="54"/>
+    </row>
+    <row r="10" spans="2:28" ht="15.6">
+      <c r="B10" s="48" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" s="51">
         <v>2</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E10" s="146" t="s">
+        <v>137</v>
+      </c>
+      <c r="E10" s="50" t="s">
+        <v>132</v>
+      </c>
+      <c r="F10" s="59" t="s">
         <v>139</v>
       </c>
-      <c r="F10" s="161" t="s">
-        <v>146</v>
-      </c>
-      <c r="G10" s="136" t="s">
-        <v>147</v>
-      </c>
-      <c r="H10" s="128" t="s">
-        <v>148</v>
+      <c r="G10" s="46" t="s">
+        <v>140</v>
+      </c>
+      <c r="H10" s="44" t="s">
+        <v>141</v>
       </c>
       <c r="I10" s="14"/>
       <c r="J10" s="14" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="K10" s="14"/>
       <c r="L10" s="14" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="M10" s="14"/>
       <c r="N10" s="14"/>
@@ -4000,250 +4067,277 @@
       <c r="P10" s="14"/>
       <c r="Q10" s="15"/>
       <c r="R10" s="15" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="S10" s="15"/>
       <c r="T10" s="15"/>
       <c r="U10" s="15"/>
-      <c r="V10" s="155" t="s">
+      <c r="V10" s="53" t="s">
+        <v>136</v>
+      </c>
+      <c r="W10" s="53"/>
+      <c r="X10" s="53"/>
+      <c r="Y10" s="53"/>
+      <c r="Z10" s="53"/>
+      <c r="AA10" s="53"/>
+      <c r="AB10" s="54"/>
+    </row>
+    <row r="11" spans="2:28" ht="15.6" customHeight="1">
+      <c r="B11" s="48" t="s">
+        <v>156</v>
+      </c>
+      <c r="C11" s="51">
+        <v>3</v>
+      </c>
+      <c r="D11" s="57" t="s">
+        <v>142</v>
+      </c>
+      <c r="E11" s="61" t="s">
         <v>143</v>
       </c>
-      <c r="W10" s="155"/>
-      <c r="X10" s="155"/>
-      <c r="Y10" s="155"/>
-      <c r="Z10" s="155"/>
-      <c r="AA10" s="155"/>
-      <c r="AB10" s="156"/>
-    </row>
-    <row r="11" spans="2:28" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="140" t="s">
-        <v>126</v>
-      </c>
-      <c r="C11" s="147">
-        <v>3</v>
-      </c>
-      <c r="D11" s="159" t="s">
-        <v>149</v>
-      </c>
-      <c r="E11" s="164" t="s">
-        <v>150</v>
-      </c>
-      <c r="F11" s="161" t="s">
-        <v>146</v>
-      </c>
-      <c r="G11" s="160" t="s">
-        <v>151</v>
-      </c>
-      <c r="H11" s="128" t="s">
-        <v>152</v>
+      <c r="F11" s="59" t="s">
+        <v>139</v>
+      </c>
+      <c r="G11" s="58" t="s">
+        <v>144</v>
+      </c>
+      <c r="H11" s="44" t="s">
+        <v>145</v>
       </c>
       <c r="I11" s="14"/>
       <c r="J11" s="14" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="K11" s="14" t="s">
-        <v>143</v>
-      </c>
-      <c r="L11" s="14"/>
+        <v>136</v>
+      </c>
+      <c r="L11" s="14" t="s">
+        <v>136</v>
+      </c>
       <c r="M11" s="14" t="s">
-        <v>143</v>
-      </c>
-      <c r="N11" s="14"/>
+        <v>136</v>
+      </c>
+      <c r="N11" s="14" t="s">
+        <v>136</v>
+      </c>
       <c r="O11" s="14"/>
       <c r="P11" s="14" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="Q11" s="15"/>
       <c r="R11" s="15"/>
       <c r="S11" s="15" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="T11" s="15"/>
       <c r="U11" s="15"/>
-      <c r="V11" s="155"/>
-      <c r="W11" s="155" t="s">
-        <v>143</v>
-      </c>
-      <c r="X11" s="155"/>
-      <c r="Y11" s="155"/>
-      <c r="Z11" s="155"/>
-      <c r="AA11" s="155"/>
-      <c r="AB11" s="156"/>
-    </row>
-    <row r="12" spans="2:28" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="140" t="s">
-        <v>127</v>
-      </c>
-      <c r="C12" s="147">
+      <c r="V11" s="53"/>
+      <c r="W11" s="53" t="s">
+        <v>136</v>
+      </c>
+      <c r="X11" s="53"/>
+      <c r="Y11" s="53"/>
+      <c r="Z11" s="53"/>
+      <c r="AA11" s="53"/>
+      <c r="AB11" s="54"/>
+    </row>
+    <row r="12" spans="2:28" ht="15.6" customHeight="1">
+      <c r="B12" s="48" t="s">
+        <v>157</v>
+      </c>
+      <c r="C12" s="51">
         <v>4</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>153</v>
-      </c>
-      <c r="E12" s="164" t="s">
-        <v>154</v>
+        <v>146</v>
+      </c>
+      <c r="E12" s="61" t="s">
+        <v>147</v>
       </c>
       <c r="F12" t="s">
-        <v>146</v>
-      </c>
-      <c r="G12" s="136" t="s">
-        <v>155</v>
-      </c>
-      <c r="H12" s="128" t="s">
-        <v>152</v>
+        <v>139</v>
+      </c>
+      <c r="G12" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="H12" s="44" t="s">
+        <v>145</v>
       </c>
       <c r="I12" s="14"/>
       <c r="J12" s="14" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="K12" s="14" t="s">
-        <v>143</v>
-      </c>
-      <c r="L12" s="14"/>
+        <v>136</v>
+      </c>
+      <c r="L12" s="14" t="s">
+        <v>136</v>
+      </c>
       <c r="M12" s="14" t="s">
-        <v>143</v>
-      </c>
-      <c r="N12" s="14"/>
+        <v>136</v>
+      </c>
+      <c r="N12" s="14" t="s">
+        <v>136</v>
+      </c>
       <c r="O12" s="14"/>
       <c r="P12" s="14" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="Q12" s="15"/>
       <c r="R12" s="15"/>
       <c r="S12" s="15" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="T12" s="15"/>
       <c r="U12" s="15"/>
-      <c r="V12" s="155"/>
-      <c r="W12" s="155"/>
-      <c r="X12" s="155" t="s">
-        <v>143</v>
-      </c>
-      <c r="Y12" s="155"/>
-      <c r="Z12" s="155"/>
-      <c r="AA12" s="155"/>
-      <c r="AB12" s="156"/>
-    </row>
-    <row r="13" spans="2:28" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="140" t="s">
-        <v>128</v>
-      </c>
-      <c r="C13" s="147">
+      <c r="V12" s="53"/>
+      <c r="W12" s="53"/>
+      <c r="X12" s="53" t="s">
+        <v>136</v>
+      </c>
+      <c r="Y12" s="53"/>
+      <c r="Z12" s="53"/>
+      <c r="AA12" s="53"/>
+      <c r="AB12" s="54"/>
+    </row>
+    <row r="13" spans="2:28" ht="15.6" customHeight="1">
+      <c r="B13" s="48" t="s">
+        <v>158</v>
+      </c>
+      <c r="C13" s="51">
         <v>5</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>156</v>
-      </c>
-      <c r="E13" s="164" t="s">
-        <v>164</v>
-      </c>
-      <c r="F13" s="161" t="s">
-        <v>146</v>
-      </c>
-      <c r="G13" s="136" t="s">
-        <v>157</v>
-      </c>
-      <c r="H13" s="128" t="s">
-        <v>158</v>
+        <v>149</v>
+      </c>
+      <c r="E13" s="61" t="s">
+        <v>183</v>
+      </c>
+      <c r="F13" s="59" t="s">
+        <v>139</v>
+      </c>
+      <c r="G13" s="46" t="s">
+        <v>184</v>
+      </c>
+      <c r="H13" s="44" t="s">
+        <v>150</v>
       </c>
       <c r="I13" s="14"/>
       <c r="J13" s="14" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="K13" s="14" t="s">
-        <v>143</v>
-      </c>
-      <c r="L13" s="14"/>
+        <v>136</v>
+      </c>
+      <c r="L13" s="14" t="s">
+        <v>136</v>
+      </c>
       <c r="M13" s="14" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="N13" s="14"/>
       <c r="O13" s="14" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="P13" s="14" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="Q13" s="15"/>
       <c r="R13" s="15"/>
       <c r="S13" s="15"/>
       <c r="T13" s="15" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="U13" s="15"/>
-      <c r="V13" s="155"/>
-      <c r="W13" s="155"/>
-      <c r="X13" s="155" t="s">
-        <v>143</v>
-      </c>
-      <c r="Y13" s="155"/>
-      <c r="Z13" s="155"/>
-      <c r="AA13" s="155"/>
-      <c r="AB13" s="156"/>
-    </row>
-    <row r="14" spans="2:28" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="141" t="s">
-        <v>129</v>
-      </c>
-      <c r="C14" s="148">
+      <c r="V13" s="53"/>
+      <c r="W13" s="53"/>
+      <c r="X13" s="53" t="s">
+        <v>136</v>
+      </c>
+      <c r="Y13" s="53"/>
+      <c r="Z13" s="53"/>
+      <c r="AA13" s="53"/>
+      <c r="AB13" s="54"/>
+    </row>
+    <row r="14" spans="2:28" ht="15.6" customHeight="1" thickBot="1">
+      <c r="B14" s="49" t="s">
+        <v>159</v>
+      </c>
+      <c r="C14" s="52">
         <v>6</v>
       </c>
-      <c r="D14" s="122" t="s">
-        <v>162</v>
-      </c>
-      <c r="E14" s="165" t="s">
-        <v>161</v>
-      </c>
-      <c r="F14" s="162" t="s">
-        <v>146</v>
-      </c>
-      <c r="G14" s="137" t="s">
-        <v>163</v>
-      </c>
-      <c r="H14" s="129" t="s">
-        <v>152</v>
-      </c>
-      <c r="I14" s="123"/>
-      <c r="J14" s="123" t="s">
-        <v>143</v>
-      </c>
-      <c r="K14" s="123" t="s">
-        <v>143</v>
-      </c>
-      <c r="L14" s="123" t="s">
-        <v>143</v>
-      </c>
-      <c r="M14" s="123" t="s">
-        <v>143</v>
-      </c>
-      <c r="N14" s="123"/>
-      <c r="O14" s="123"/>
-      <c r="P14" s="123" t="s">
-        <v>143</v>
-      </c>
-      <c r="Q14" s="124"/>
-      <c r="R14" s="124"/>
-      <c r="S14" s="124"/>
-      <c r="T14" s="124"/>
-      <c r="U14" s="124" t="s">
-        <v>143</v>
-      </c>
-      <c r="V14" s="157"/>
-      <c r="W14" s="157" t="s">
-        <v>143</v>
-      </c>
-      <c r="X14" s="157"/>
-      <c r="Y14" s="157"/>
-      <c r="Z14" s="157"/>
-      <c r="AA14" s="157"/>
-      <c r="AB14" s="158"/>
-    </row>
-    <row r="15" spans="2:28" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D14" s="41" t="s">
+        <v>154</v>
+      </c>
+      <c r="E14" s="62" t="s">
+        <v>153</v>
+      </c>
+      <c r="F14" s="60" t="s">
+        <v>139</v>
+      </c>
+      <c r="G14" s="47" t="s">
+        <v>155</v>
+      </c>
+      <c r="H14" s="45" t="s">
+        <v>145</v>
+      </c>
+      <c r="I14" s="42"/>
+      <c r="J14" s="42" t="s">
+        <v>136</v>
+      </c>
+      <c r="K14" s="42" t="s">
+        <v>136</v>
+      </c>
+      <c r="L14" s="42" t="s">
+        <v>136</v>
+      </c>
+      <c r="M14" s="42" t="s">
+        <v>136</v>
+      </c>
+      <c r="N14" s="42" t="s">
+        <v>136</v>
+      </c>
+      <c r="O14" s="42"/>
+      <c r="P14" s="42" t="s">
+        <v>136</v>
+      </c>
+      <c r="Q14" s="43"/>
+      <c r="R14" s="43"/>
+      <c r="S14" s="43"/>
+      <c r="T14" s="43"/>
+      <c r="U14" s="43" t="s">
+        <v>136</v>
+      </c>
+      <c r="V14" s="55"/>
+      <c r="W14" s="55" t="s">
+        <v>136</v>
+      </c>
+      <c r="X14" s="55"/>
+      <c r="Y14" s="55"/>
+      <c r="Z14" s="55"/>
+      <c r="AA14" s="55"/>
+      <c r="AB14" s="56"/>
+    </row>
+    <row r="15" spans="2:28" ht="15.6">
       <c r="B15" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="B5:B8"/>
+    <mergeCell ref="Z7:Z8"/>
+    <mergeCell ref="AA7:AA8"/>
+    <mergeCell ref="G7:G8"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="W7:W8"/>
+    <mergeCell ref="X7:X8"/>
+    <mergeCell ref="Y7:Y8"/>
+    <mergeCell ref="U7:U8"/>
+    <mergeCell ref="V6:AB6"/>
+    <mergeCell ref="Q7:Q8"/>
+    <mergeCell ref="R7:R8"/>
+    <mergeCell ref="S7:S8"/>
+    <mergeCell ref="T7:T8"/>
+    <mergeCell ref="D1:G1"/>
     <mergeCell ref="Q6:U6"/>
     <mergeCell ref="H5:AB5"/>
     <mergeCell ref="B3:G3"/>
@@ -4260,21 +4354,6 @@
     <mergeCell ref="M7:N7"/>
     <mergeCell ref="O7:P7"/>
     <mergeCell ref="V7:V8"/>
-    <mergeCell ref="Q7:Q8"/>
-    <mergeCell ref="R7:R8"/>
-    <mergeCell ref="S7:S8"/>
-    <mergeCell ref="T7:T8"/>
-    <mergeCell ref="D1:G1"/>
-    <mergeCell ref="B5:B8"/>
-    <mergeCell ref="Z7:Z8"/>
-    <mergeCell ref="AA7:AA8"/>
-    <mergeCell ref="G7:G8"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="W7:W8"/>
-    <mergeCell ref="X7:X8"/>
-    <mergeCell ref="Y7:Y8"/>
-    <mergeCell ref="U7:U8"/>
-    <mergeCell ref="V6:AB6"/>
   </mergeCells>
   <phoneticPr fontId="17" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4288,270 +4367,266 @@
     <tabColor theme="3" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="B1:N17"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="3" max="3" width="7.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="31.44140625" customWidth="1"/>
+    <col min="5" max="5" width="13.109375" customWidth="1"/>
     <col min="6" max="6" width="34.6640625" customWidth="1"/>
-    <col min="7" max="7" width="23.77734375" customWidth="1"/>
+    <col min="7" max="7" width="31" customWidth="1"/>
     <col min="8" max="8" width="22.21875" customWidth="1"/>
-    <col min="10" max="10" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.109375" customWidth="1"/>
+    <col min="9" max="9" width="53.77734375" customWidth="1"/>
+    <col min="10" max="10" width="57.109375" customWidth="1"/>
+    <col min="11" max="11" width="48.88671875" customWidth="1"/>
     <col min="12" max="12" width="18.44140625" customWidth="1"/>
     <col min="13" max="13" width="25.44140625" customWidth="1"/>
     <col min="15" max="15" width="12.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:14">
       <c r="B1" s="11"/>
-      <c r="D1" s="35" t="s">
+      <c r="D1" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="37"/>
-    </row>
-    <row r="3" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B3" s="54" t="s">
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="67"/>
+    </row>
+    <row r="3" spans="2:14">
+      <c r="B3" s="169" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3" s="170"/>
+      <c r="D3" s="170"/>
+      <c r="E3" s="170"/>
+      <c r="F3" s="170"/>
+      <c r="G3" s="170"/>
+      <c r="H3" s="170"/>
+      <c r="I3" s="170"/>
+      <c r="J3" s="170"/>
+      <c r="K3" s="171"/>
+    </row>
+    <row r="4" spans="2:14">
+      <c r="B4" s="156" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" s="151" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" s="162" t="s">
         <v>50</v>
       </c>
-      <c r="C3" s="54"/>
-      <c r="D3" s="54"/>
-      <c r="E3" s="54"/>
-      <c r="F3" s="54"/>
-      <c r="G3" s="54"/>
-      <c r="H3" s="54"/>
-      <c r="I3" s="54"/>
-      <c r="J3" s="54"/>
-      <c r="K3" s="54"/>
-      <c r="L3" s="54"/>
-    </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B4" s="55" t="s">
+      <c r="E4" s="158" t="s">
         <v>51</v>
       </c>
-      <c r="C4" s="64" t="s">
+      <c r="F4" s="160"/>
+      <c r="G4" s="160"/>
+      <c r="H4" s="160"/>
+      <c r="I4" s="159"/>
+      <c r="J4" s="158" t="s">
         <v>52</v>
       </c>
-      <c r="D4" s="66" t="s">
+      <c r="K4" s="159"/>
+    </row>
+    <row r="5" spans="2:14" ht="15" customHeight="1" thickBot="1">
+      <c r="B5" s="157"/>
+      <c r="C5" s="161"/>
+      <c r="D5" s="163"/>
+      <c r="E5" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="I5" s="36" t="s">
+        <v>161</v>
+      </c>
+      <c r="J5" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E4" s="57" t="s">
+      <c r="K5" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="F4" s="63"/>
-      <c r="G4" s="63"/>
-      <c r="H4" s="63"/>
-      <c r="I4" s="63"/>
-      <c r="J4" s="58"/>
-      <c r="K4" s="57" t="s">
-        <v>55</v>
-      </c>
-      <c r="L4" s="58"/>
-    </row>
-    <row r="5" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="56"/>
-      <c r="C5" s="65"/>
-      <c r="D5" s="67"/>
-      <c r="E5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" s="59" t="s">
-        <v>20</v>
-      </c>
-      <c r="J5" s="60"/>
-      <c r="K5" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="6" spans="2:14" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="2:14" ht="15" customHeight="1" thickTop="1">
       <c r="B6" s="17">
         <v>1</v>
       </c>
-      <c r="C6" s="169" t="s">
-        <v>58</v>
+      <c r="C6" s="131" t="s">
+        <v>55</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="E6" s="18" t="s">
-        <v>20</v>
+        <v>46</v>
+      </c>
+      <c r="E6" s="18">
+        <v>1</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>20</v>
+        <v>138</v>
       </c>
       <c r="G6" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="H6" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="I6" s="68" t="s">
-        <v>20</v>
-      </c>
-      <c r="J6" s="69"/>
-      <c r="K6" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="L6" s="17" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.3">
+        <v>132</v>
+      </c>
+      <c r="H6" s="166" t="s">
+        <v>162</v>
+      </c>
+      <c r="I6" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="J6" s="18" t="s">
+        <v>171</v>
+      </c>
+      <c r="K6" s="17" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="7" spans="2:14">
       <c r="B7" s="17">
         <v>2</v>
       </c>
-      <c r="C7" s="61"/>
+      <c r="C7" s="132"/>
       <c r="D7" s="4" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E7" s="17">
-        <v>5</v>
-      </c>
-      <c r="F7" s="17">
-        <v>6</v>
+        <v>2</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>137</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="H7" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="I7" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="J7" s="58"/>
+        <v>132</v>
+      </c>
+      <c r="H7" s="167"/>
+      <c r="I7" s="35" t="s">
+        <v>179</v>
+      </c>
+      <c r="J7" s="17" t="s">
+        <v>172</v>
+      </c>
       <c r="K7" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="L7" s="17" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.3">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="8" spans="2:14">
       <c r="B8" s="17">
         <v>3</v>
       </c>
-      <c r="C8" s="61"/>
+      <c r="C8" s="132"/>
       <c r="D8" s="10" t="s">
-        <v>165</v>
-      </c>
-      <c r="E8" s="17" t="s">
-        <v>20</v>
+        <v>156</v>
+      </c>
+      <c r="E8" s="17">
+        <v>3</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="H8" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="I8" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="J8" s="58"/>
+        <v>143</v>
+      </c>
+      <c r="H8" s="167"/>
+      <c r="I8" s="35" t="s">
+        <v>178</v>
+      </c>
+      <c r="J8" s="17" t="s">
+        <v>173</v>
+      </c>
       <c r="K8" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="L8" s="17" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.3">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="9" spans="2:14">
       <c r="B9" s="17">
         <v>4</v>
       </c>
-      <c r="C9" s="61"/>
+      <c r="C9" s="132"/>
       <c r="D9" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="E9" s="17">
+        <v>4</v>
+      </c>
+      <c r="F9" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="G9" s="17" t="s">
+        <v>181</v>
+      </c>
+      <c r="H9" s="167"/>
+      <c r="I9" s="35" t="s">
+        <v>177</v>
+      </c>
+      <c r="J9" s="17" t="s">
+        <v>174</v>
+      </c>
+      <c r="K9" s="17" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="10" spans="2:14">
+      <c r="B10" s="63">
+        <v>5</v>
+      </c>
+      <c r="C10" s="132"/>
+      <c r="D10" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="E10" s="63">
+        <v>5</v>
+      </c>
+      <c r="F10" s="63" t="s">
+        <v>149</v>
+      </c>
+      <c r="G10" s="63" t="s">
+        <v>182</v>
+      </c>
+      <c r="H10" s="167"/>
+      <c r="I10" s="64" t="s">
+        <v>176</v>
+      </c>
+      <c r="J10" s="63" t="s">
+        <v>175</v>
+      </c>
+      <c r="K10" s="63" t="s">
         <v>166</v>
       </c>
-      <c r="E9" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="F9" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="G9" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="H9" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="I9" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="J9" s="58"/>
-      <c r="K9" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="L9" s="17" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B10" s="166">
-        <v>5</v>
-      </c>
-      <c r="C10" s="61"/>
-      <c r="D10" s="10" t="s">
-        <v>167</v>
-      </c>
-      <c r="E10" s="166"/>
-      <c r="F10" s="166"/>
-      <c r="G10" s="166"/>
-      <c r="H10" s="166"/>
-      <c r="I10" s="168"/>
-      <c r="J10" s="167"/>
-      <c r="K10" s="166"/>
-      <c r="L10" s="166"/>
-    </row>
-    <row r="11" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="11" spans="2:14" ht="15" thickBot="1">
       <c r="B11" s="2">
         <v>6</v>
       </c>
-      <c r="C11" s="62"/>
+      <c r="C11" s="133"/>
       <c r="D11" s="9" t="s">
-        <v>168</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>20</v>
+        <v>159</v>
+      </c>
+      <c r="E11" s="2">
+        <v>6</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>20</v>
+        <v>154</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I11" s="59" t="s">
-        <v>20</v>
-      </c>
-      <c r="J11" s="60"/>
+        <v>185</v>
+      </c>
+      <c r="H11" s="168"/>
+      <c r="I11" s="36" t="s">
+        <v>163</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>164</v>
+      </c>
       <c r="K11" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="L11" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="2:14" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="12" spans="2:14" ht="15" thickTop="1">
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
@@ -4564,92 +4639,92 @@
       <c r="K12" s="3"/>
       <c r="L12" s="3"/>
     </row>
-    <row r="13" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:14" ht="15" thickBot="1">
       <c r="B13" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="K13" s="19"/>
+    </row>
+    <row r="14" spans="2:14" ht="15.6" thickTop="1" thickBot="1">
+      <c r="B14" s="134" t="s">
+        <v>58</v>
+      </c>
+      <c r="C14" s="135"/>
+      <c r="D14" s="135"/>
+      <c r="E14" s="135"/>
+      <c r="F14" s="164" t="s">
+        <v>59</v>
+      </c>
+      <c r="G14" s="165"/>
+      <c r="H14" s="134" t="s">
         <v>60</v>
       </c>
-      <c r="K13" s="19"/>
-    </row>
-    <row r="14" spans="2:14" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="52" t="s">
+      <c r="I14" s="135"/>
+      <c r="J14" s="135"/>
+      <c r="K14" s="135"/>
+      <c r="L14" s="136"/>
+      <c r="M14" s="141" t="s">
         <v>61</v>
       </c>
-      <c r="C14" s="53"/>
-      <c r="D14" s="53"/>
-      <c r="E14" s="53"/>
-      <c r="F14" s="70" t="s">
+      <c r="N14" s="142"/>
+    </row>
+    <row r="15" spans="2:14" ht="15" thickTop="1">
+      <c r="B15" s="140" t="s">
         <v>62</v>
       </c>
-      <c r="G14" s="71"/>
-      <c r="H14" s="52" t="s">
+      <c r="C15" s="144" t="s">
         <v>63</v>
       </c>
-      <c r="I14" s="53"/>
-      <c r="J14" s="53"/>
-      <c r="K14" s="53"/>
-      <c r="L14" s="80"/>
-      <c r="M14" s="85" t="s">
+      <c r="D15" s="144" t="s">
         <v>64</v>
       </c>
-      <c r="N14" s="86"/>
-    </row>
-    <row r="15" spans="2:14" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="84" t="s">
+      <c r="E15" s="146" t="s">
         <v>65</v>
       </c>
-      <c r="C15" s="76" t="s">
+      <c r="F15" s="148" t="s">
         <v>66</v>
       </c>
-      <c r="D15" s="76" t="s">
+      <c r="G15" s="150" t="s">
         <v>67</v>
       </c>
-      <c r="E15" s="88" t="s">
+      <c r="H15" s="152" t="s">
         <v>68</v>
       </c>
-      <c r="F15" s="73" t="s">
+      <c r="I15" s="144" t="s">
+        <v>62</v>
+      </c>
+      <c r="J15" s="144" t="s">
+        <v>63</v>
+      </c>
+      <c r="K15" s="154" t="s">
         <v>69</v>
       </c>
-      <c r="G15" s="72" t="s">
+      <c r="L15" s="137" t="s">
         <v>70</v>
       </c>
-      <c r="H15" s="74" t="s">
+      <c r="M15" s="139" t="s">
         <v>71</v>
       </c>
-      <c r="I15" s="76" t="s">
-        <v>65</v>
-      </c>
-      <c r="J15" s="76" t="s">
-        <v>66</v>
-      </c>
-      <c r="K15" s="78" t="s">
+      <c r="N15" s="151" t="s">
         <v>72</v>
       </c>
-      <c r="L15" s="81" t="s">
-        <v>73</v>
-      </c>
-      <c r="M15" s="83" t="s">
-        <v>74</v>
-      </c>
-      <c r="N15" s="64" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B16" s="87"/>
-      <c r="C16" s="77"/>
-      <c r="D16" s="77"/>
-      <c r="E16" s="89"/>
-      <c r="F16" s="90"/>
-      <c r="G16" s="72"/>
-      <c r="H16" s="75"/>
-      <c r="I16" s="77"/>
-      <c r="J16" s="77"/>
-      <c r="K16" s="79"/>
-      <c r="L16" s="82"/>
-      <c r="M16" s="84"/>
-      <c r="N16" s="73"/>
-    </row>
-    <row r="17" spans="2:14" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="2:14">
+      <c r="B16" s="143"/>
+      <c r="C16" s="145"/>
+      <c r="D16" s="145"/>
+      <c r="E16" s="147"/>
+      <c r="F16" s="149"/>
+      <c r="G16" s="150"/>
+      <c r="H16" s="153"/>
+      <c r="I16" s="145"/>
+      <c r="J16" s="145"/>
+      <c r="K16" s="155"/>
+      <c r="L16" s="138"/>
+      <c r="M16" s="140"/>
+      <c r="N16" s="148"/>
+    </row>
+    <row r="17" spans="2:14">
       <c r="B17" s="23">
         <v>6</v>
       </c>
@@ -4666,10 +4741,10 @@
         <v>0</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="I17" s="23">
         <f>SUM(J17:K17)</f>
@@ -4683,25 +4758,31 @@
       </c>
       <c r="L17" s="25"/>
       <c r="M17" s="6" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="N17" s="26">
-        <f>C17</f>
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="31">
+  <mergeCells count="26">
+    <mergeCell ref="D1:G1"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:I4"/>
+    <mergeCell ref="B3:K3"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="F15:F16"/>
     <mergeCell ref="C6:C11"/>
     <mergeCell ref="H14:L14"/>
     <mergeCell ref="L15:L16"/>
     <mergeCell ref="M15:M16"/>
     <mergeCell ref="M14:N14"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="F15:F16"/>
     <mergeCell ref="G15:G16"/>
     <mergeCell ref="N15:N16"/>
     <mergeCell ref="H15:H16"/>
@@ -4709,20 +4790,8 @@
     <mergeCell ref="K15:K16"/>
     <mergeCell ref="J15:J16"/>
     <mergeCell ref="B14:E14"/>
-    <mergeCell ref="D1:G1"/>
-    <mergeCell ref="B3:L3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="E4:J4"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="I8:J8"/>
     <mergeCell ref="F14:G14"/>
+    <mergeCell ref="H6:H11"/>
   </mergeCells>
   <phoneticPr fontId="17" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4731,6 +4800,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E819BB071F23F542A5DF0E9C9037AD04" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="798a38e6de461387c626d04793181ea9">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="301f98df-4edd-4096-94f8-2f8af3eee570" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b4b8dab68acb31e3ac71f6347d499c29" ns2:_="">
     <xsd:import namespace="301f98df-4edd-4096-94f8-2f8af3eee570"/>
@@ -4868,12 +4943,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -4884,6 +4953,15 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA2F5940-EC19-4D08-A8C2-FA31EF734077}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A94B7F00-F329-4E8F-A3EE-411E39CDE676}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4901,15 +4979,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA2F5940-EC19-4D08-A8C2-FA31EF734077}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EECFCB93-350B-4228-B7F4-DB12383611F2}">
   <ds:schemaRefs>

</xml_diff>